<commit_message>
data: update NA Bench Forecast — 2026-08-12 12:17
</commit_message>
<xml_diff>
--- a/NA Bench Forecast.xlsx
+++ b/NA Bench Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbondcrx/Desktop/BOB!/Bench Forecast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49377630-B33A-E340-8802-9DB5AB916347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6740DF-130B-A347-A39C-345F93944A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="2520" windowWidth="27320" windowHeight="16080" xr2:uid="{25195C4B-21BA-C647-88E3-DB4384B68E18}"/>
+    <workbookView xWindow="1200" yWindow="1740" windowWidth="27320" windowHeight="16080" xr2:uid="{25195C4B-21BA-C647-88E3-DB4384B68E18}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench Forecast" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,8 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="438" r:id="rId8"/>
-    <pivotCache cacheId="442" r:id="rId9"/>
+    <pivotCache cacheId="528" r:id="rId8"/>
+    <pivotCache cacheId="529" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -888,7 +888,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1002,14 +1002,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1019,12 +1014,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1572,43 +1569,43 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>7.0541480377545956E-2</c:v>
+                  <c:v>6.8554396423248884E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>7.6999503229011432E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>7.7993045206159961E-2</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
+                  <c:v>7.9483358171882762E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>7.9980129160457034E-2</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.3457526080476907E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8.2463984103328364E-2</c:v>
-                </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.9418777943368111E-2</c:v>
+                  <c:v>8.2960755091902635E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.9915548931942368E-2</c:v>
+                  <c:v>8.2960755091902635E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8.9418777943368111E-2</c:v>
+                  <c:v>8.2960755091902635E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.8425235966219567E-2</c:v>
+                  <c:v>8.5444610034773966E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.10531544957774466</c:v>
+                  <c:v>0.10382513661202186</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.11028315946348734</c:v>
+                  <c:v>0.10879284649776454</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.11028315946348734</c:v>
+                  <c:v>0.10779930452061599</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.10829607550919026</c:v>
+                  <c:v>0.10581222056631892</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18347,7 +18344,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EBC7B274-FD7A-844F-964F-72EF841A0267}" name="PivotTable12" cacheId="438" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EBC7B274-FD7A-844F-964F-72EF841A0267}" name="PivotTable12" cacheId="528" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
   <location ref="Q23:R107" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
@@ -18814,7 +18811,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{04DCFBA1-C6D5-3C43-8822-30BD597F8EAC}" name="PivotTable2" cacheId="442" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="43">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{04DCFBA1-C6D5-3C43-8822-30BD597F8EAC}" name="PivotTable2" cacheId="529" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="43">
   <location ref="A36:E50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisCol" showAll="0">
@@ -20556,43 +20553,43 @@
         <v>20</v>
       </c>
       <c r="B8" s="12">
+        <v>20</v>
+      </c>
+      <c r="C8" s="12">
+        <v>22</v>
+      </c>
+      <c r="D8" s="12">
         <v>24</v>
       </c>
-      <c r="C8" s="12">
+      <c r="E8" s="12">
+        <v>23</v>
+      </c>
+      <c r="F8" s="12">
         <v>24</v>
       </c>
-      <c r="D8" s="12">
-        <v>28</v>
-      </c>
-      <c r="E8" s="12">
-        <v>31</v>
-      </c>
-      <c r="F8" s="12">
-        <v>29</v>
-      </c>
       <c r="G8" s="12">
+        <v>20</v>
+      </c>
+      <c r="H8" s="8">
+        <v>19</v>
+      </c>
+      <c r="I8" s="8">
+        <v>20</v>
+      </c>
+      <c r="J8" s="8">
+        <v>27</v>
+      </c>
+      <c r="K8" s="8">
         <v>33</v>
       </c>
-      <c r="H8" s="8">
+      <c r="L8" s="8">
         <v>33</v>
       </c>
-      <c r="I8" s="8">
+      <c r="M8" s="8">
         <v>33</v>
       </c>
-      <c r="J8" s="8">
+      <c r="N8" s="8">
         <v>33</v>
-      </c>
-      <c r="K8" s="8">
-        <v>36</v>
-      </c>
-      <c r="L8" s="8">
-        <v>36</v>
-      </c>
-      <c r="M8" s="8">
-        <v>38</v>
-      </c>
-      <c r="N8" s="8">
-        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -20601,55 +20598,55 @@
       </c>
       <c r="B9" s="6">
         <f>SUM(B2:B8)</f>
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C9" s="6">
         <f t="shared" ref="C9:N9" si="0">SUM(C2:C8)</f>
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D9" s="6">
         <f t="shared" si="0"/>
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E9" s="6">
         <f t="shared" si="0"/>
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="F9" s="6">
         <f t="shared" si="0"/>
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="G9" s="6">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="H9" s="6">
         <f t="shared" si="0"/>
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="J9" s="6">
         <f t="shared" si="0"/>
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="K9" s="6">
         <f t="shared" si="0"/>
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="L9" s="6">
         <f t="shared" si="0"/>
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="M9" s="6">
         <f t="shared" si="0"/>
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="N9" s="6">
         <f t="shared" si="0"/>
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -20658,55 +20655,55 @@
       </c>
       <c r="B10" s="7">
         <f>+B9/$B$11</f>
-        <v>7.0541480377545956E-2</v>
+        <v>6.8554396423248884E-2</v>
       </c>
       <c r="C10" s="7">
         <f t="shared" ref="C10:N10" si="1">+C9/$B$11</f>
-        <v>7.7993045206159961E-2</v>
+        <v>7.6999503229011432E-2</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9980129160457034E-2</v>
+        <v>7.7993045206159961E-2</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="1"/>
-        <v>8.3457526080476907E-2</v>
+        <v>7.9483358171882762E-2</v>
       </c>
       <c r="F10" s="7">
         <f t="shared" si="1"/>
-        <v>8.2463984103328364E-2</v>
+        <v>7.9980129160457034E-2</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" si="1"/>
-        <v>8.9418777943368111E-2</v>
+        <v>8.2960755091902635E-2</v>
       </c>
       <c r="H10" s="7">
         <f t="shared" si="1"/>
-        <v>8.9915548931942368E-2</v>
+        <v>8.2960755091902635E-2</v>
       </c>
       <c r="I10" s="7">
         <f t="shared" si="1"/>
-        <v>8.9418777943368111E-2</v>
+        <v>8.2960755091902635E-2</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="1"/>
-        <v>8.8425235966219567E-2</v>
+        <v>8.5444610034773966E-2</v>
       </c>
       <c r="K10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10531544957774466</v>
+        <v>0.10382513661202186</v>
       </c>
       <c r="L10" s="7">
         <f t="shared" si="1"/>
-        <v>0.11028315946348734</v>
+        <v>0.10879284649776454</v>
       </c>
       <c r="M10" s="7">
         <f t="shared" si="1"/>
-        <v>0.11028315946348734</v>
+        <v>0.10779930452061599</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10829607550919026</v>
+        <v>0.10581222056631892</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -25242,149 +25239,149 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="21"/>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
-      <c r="V1" s="42"/>
-      <c r="W1" s="42"/>
-      <c r="X1" s="42"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="42"/>
-      <c r="AA1" s="42"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="46"/>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="46"/>
+      <c r="S1" s="46"/>
+      <c r="T1" s="46"/>
+      <c r="U1" s="46"/>
+      <c r="V1" s="46"/>
+      <c r="W1" s="46"/>
+      <c r="X1" s="46"/>
+      <c r="Y1" s="46"/>
+      <c r="Z1" s="46"/>
+      <c r="AA1" s="46"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="44" t="s">
+      <c r="C2" s="43"/>
+      <c r="D2" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="45"/>
-      <c r="F2" s="44" t="s">
+      <c r="E2" s="43"/>
+      <c r="F2" s="42" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="45"/>
-      <c r="H2" s="44" t="s">
+      <c r="G2" s="43"/>
+      <c r="H2" s="42" t="s">
         <v>131</v>
       </c>
-      <c r="I2" s="45"/>
-      <c r="J2" s="44" t="s">
+      <c r="I2" s="43"/>
+      <c r="J2" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="K2" s="45"/>
-      <c r="L2" s="44" t="s">
+      <c r="K2" s="43"/>
+      <c r="L2" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="M2" s="45"/>
-      <c r="N2" s="44" t="s">
+      <c r="M2" s="43"/>
+      <c r="N2" s="42" t="s">
         <v>134</v>
       </c>
-      <c r="O2" s="45"/>
-      <c r="P2" s="44" t="s">
+      <c r="O2" s="43"/>
+      <c r="P2" s="42" t="s">
         <v>135</v>
       </c>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="44" t="s">
+      <c r="Q2" s="43"/>
+      <c r="R2" s="42" t="s">
         <v>136</v>
       </c>
-      <c r="S2" s="45"/>
-      <c r="T2" s="44" t="s">
+      <c r="S2" s="43"/>
+      <c r="T2" s="42" t="s">
         <v>137</v>
       </c>
-      <c r="U2" s="45"/>
-      <c r="V2" s="44" t="s">
+      <c r="U2" s="43"/>
+      <c r="V2" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="W2" s="45"/>
-      <c r="X2" s="44" t="s">
+      <c r="W2" s="43"/>
+      <c r="X2" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="Y2" s="45"/>
-      <c r="Z2" s="44" t="s">
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="42" t="s">
         <v>140</v>
       </c>
-      <c r="AA2" s="45"/>
+      <c r="AA2" s="43"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="43"/>
-      <c r="B3" s="44" t="s">
+      <c r="A3" s="44"/>
+      <c r="B3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="44" t="s">
+      <c r="C3" s="43"/>
+      <c r="D3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="44" t="s">
+      <c r="E3" s="43"/>
+      <c r="F3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="44" t="s">
+      <c r="G3" s="43"/>
+      <c r="H3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="I3" s="45"/>
-      <c r="J3" s="44" t="s">
+      <c r="I3" s="43"/>
+      <c r="J3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="K3" s="45"/>
-      <c r="L3" s="44" t="s">
+      <c r="K3" s="43"/>
+      <c r="L3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="M3" s="45"/>
-      <c r="N3" s="44" t="s">
+      <c r="M3" s="43"/>
+      <c r="N3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="O3" s="45"/>
-      <c r="P3" s="44" t="s">
+      <c r="O3" s="43"/>
+      <c r="P3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="Q3" s="45"/>
-      <c r="R3" s="44" t="s">
+      <c r="Q3" s="43"/>
+      <c r="R3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="S3" s="45"/>
-      <c r="T3" s="44" t="s">
+      <c r="S3" s="43"/>
+      <c r="T3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="U3" s="45"/>
-      <c r="V3" s="44" t="s">
+      <c r="U3" s="43"/>
+      <c r="V3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="W3" s="45"/>
-      <c r="X3" s="44" t="s">
+      <c r="W3" s="43"/>
+      <c r="X3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="44" t="s">
+      <c r="Y3" s="43"/>
+      <c r="Z3" s="42" t="s">
         <v>141</v>
       </c>
-      <c r="AA3" s="45"/>
+      <c r="AA3" s="43"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="43"/>
+      <c r="A4" s="44"/>
       <c r="B4" s="23" t="s">
         <v>142</v>
       </c>
@@ -26129,7 +26126,7 @@
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A15" s="43" t="s">
+      <c r="A15" s="44" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="22" t="s">
@@ -26172,21 +26169,21 @@
         <v>140</v>
       </c>
       <c r="O15" s="36"/>
-      <c r="P15" s="46"/>
-      <c r="Q15" s="46"/>
-      <c r="R15" s="46"/>
-      <c r="S15" s="46"/>
-      <c r="T15" s="46"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="46"/>
-      <c r="W15" s="46"/>
-      <c r="X15" s="46"/>
-      <c r="Y15" s="46"/>
-      <c r="Z15" s="46"/>
-      <c r="AA15" s="46"/>
+      <c r="P15" s="41"/>
+      <c r="Q15" s="41"/>
+      <c r="R15" s="41"/>
+      <c r="S15" s="41"/>
+      <c r="T15" s="41"/>
+      <c r="U15" s="41"/>
+      <c r="V15" s="41"/>
+      <c r="W15" s="41"/>
+      <c r="X15" s="41"/>
+      <c r="Y15" s="41"/>
+      <c r="Z15" s="41"/>
+      <c r="AA15" s="41"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A16" s="43"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="23" t="s">
         <v>143</v>
       </c>
@@ -26857,55 +26854,55 @@
       </c>
       <c r="B31" s="1">
         <f>+'Bench Forecast'!B9</f>
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C31" s="1">
         <f>+'Bench Forecast'!C9</f>
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D31" s="1">
         <f>+'Bench Forecast'!D9</f>
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E31" s="1">
         <f>+'Bench Forecast'!E9</f>
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="F31" s="1">
         <f>+'Bench Forecast'!F9</f>
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="G31" s="1">
         <f>+'Bench Forecast'!G9</f>
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="H31" s="1">
         <f>+'Bench Forecast'!H9</f>
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="I31" s="1">
         <f>+'Bench Forecast'!I9</f>
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="J31" s="1">
         <f>+'Bench Forecast'!J9</f>
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="K31" s="1">
         <f>+'Bench Forecast'!K9</f>
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="L31" s="1">
         <f>+'Bench Forecast'!L9</f>
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="M31" s="1">
         <f>+'Bench Forecast'!M9</f>
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="N31" s="1">
         <f>+'Bench Forecast'!N9</f>
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.2">
@@ -27038,16 +27035,16 @@
       <c r="A38" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B38" s="47">
+      <c r="B38" s="1">
         <v>142</v>
       </c>
-      <c r="C38" s="47">
+      <c r="C38" s="1">
         <v>159</v>
       </c>
-      <c r="D38" s="47">
+      <c r="D38" s="1">
         <v>159</v>
       </c>
-      <c r="E38" s="47">
+      <c r="E38" s="1">
         <v>460</v>
       </c>
     </row>
@@ -27055,16 +27052,16 @@
       <c r="A39" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B39" s="47">
+      <c r="B39" s="1">
         <v>157</v>
       </c>
-      <c r="C39" s="47">
+      <c r="C39" s="1">
         <v>148</v>
       </c>
-      <c r="D39" s="47">
+      <c r="D39" s="1">
         <v>161</v>
       </c>
-      <c r="E39" s="47">
+      <c r="E39" s="1">
         <v>466</v>
       </c>
     </row>
@@ -27072,16 +27069,16 @@
       <c r="A40" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B40" s="47">
+      <c r="B40" s="1">
         <v>161</v>
       </c>
-      <c r="C40" s="47">
+      <c r="C40" s="1">
         <v>133</v>
       </c>
-      <c r="D40" s="47">
+      <c r="D40" s="1">
         <v>154</v>
       </c>
-      <c r="E40" s="47">
+      <c r="E40" s="1">
         <v>448</v>
       </c>
     </row>
@@ -27089,16 +27086,16 @@
       <c r="A41" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B41" s="47">
+      <c r="B41" s="1">
         <v>168</v>
       </c>
-      <c r="C41" s="47">
+      <c r="C41" s="1">
         <v>138</v>
       </c>
-      <c r="D41" s="47">
+      <c r="D41" s="1">
         <v>156</v>
       </c>
-      <c r="E41" s="47">
+      <c r="E41" s="1">
         <v>462</v>
       </c>
     </row>
@@ -27106,16 +27103,16 @@
       <c r="A42" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B42" s="47">
+      <c r="B42" s="1">
         <v>166</v>
       </c>
-      <c r="C42" s="47">
+      <c r="C42" s="1">
         <v>121</v>
       </c>
-      <c r="D42" s="47">
+      <c r="D42" s="1">
         <v>152</v>
       </c>
-      <c r="E42" s="47">
+      <c r="E42" s="1">
         <v>439</v>
       </c>
     </row>
@@ -27123,16 +27120,16 @@
       <c r="A43" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B43" s="47">
+      <c r="B43" s="1">
         <v>180</v>
       </c>
-      <c r="C43" s="47">
+      <c r="C43" s="1">
         <v>136</v>
       </c>
-      <c r="D43" s="47">
+      <c r="D43" s="1">
         <v>165</v>
       </c>
-      <c r="E43" s="47">
+      <c r="E43" s="1">
         <v>481</v>
       </c>
     </row>
@@ -27140,16 +27137,16 @@
       <c r="A44" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B44" s="47">
+      <c r="B44" s="1">
         <v>181</v>
       </c>
-      <c r="C44" s="47">
+      <c r="C44" s="1">
         <v>119</v>
       </c>
-      <c r="D44" s="47">
+      <c r="D44" s="1">
         <v>175</v>
       </c>
-      <c r="E44" s="47">
+      <c r="E44" s="1">
         <v>475</v>
       </c>
     </row>
@@ -27157,16 +27154,16 @@
       <c r="A45" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B45" s="47">
+      <c r="B45" s="1">
         <v>180</v>
       </c>
-      <c r="C45" s="47">
+      <c r="C45" s="1">
         <v>114</v>
       </c>
-      <c r="D45" s="47">
+      <c r="D45" s="1">
         <v>176</v>
       </c>
-      <c r="E45" s="47">
+      <c r="E45" s="1">
         <v>470</v>
       </c>
     </row>
@@ -27174,16 +27171,16 @@
       <c r="A46" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B46" s="47">
+      <c r="B46" s="1">
         <v>178</v>
       </c>
-      <c r="C46" s="47">
+      <c r="C46" s="1">
         <v>104</v>
       </c>
-      <c r="D46" s="47">
+      <c r="D46" s="1">
         <v>171</v>
       </c>
-      <c r="E46" s="47">
+      <c r="E46" s="1">
         <v>453</v>
       </c>
     </row>
@@ -27191,16 +27188,16 @@
       <c r="A47" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B47" s="47">
+      <c r="B47" s="1">
         <v>212</v>
       </c>
-      <c r="C47" s="47">
+      <c r="C47" s="1">
         <v>112</v>
       </c>
-      <c r="D47" s="47">
+      <c r="D47" s="1">
         <v>196</v>
       </c>
-      <c r="E47" s="47">
+      <c r="E47" s="1">
         <v>520</v>
       </c>
     </row>
@@ -27208,16 +27205,16 @@
       <c r="A48" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B48" s="47">
+      <c r="B48" s="1">
         <v>222</v>
       </c>
-      <c r="C48" s="47">
+      <c r="C48" s="1">
         <v>98</v>
       </c>
-      <c r="D48" s="47">
+      <c r="D48" s="1">
         <v>192</v>
       </c>
-      <c r="E48" s="47">
+      <c r="E48" s="1">
         <v>512</v>
       </c>
     </row>
@@ -27225,16 +27222,16 @@
       <c r="A49" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B49" s="47">
+      <c r="B49" s="1">
         <v>222</v>
       </c>
-      <c r="C49" s="47">
+      <c r="C49" s="1">
         <v>95</v>
       </c>
-      <c r="D49" s="47">
+      <c r="D49" s="1">
         <v>191</v>
       </c>
-      <c r="E49" s="47">
+      <c r="E49" s="1">
         <v>508</v>
       </c>
     </row>
@@ -27242,26 +27239,36 @@
       <c r="A50" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B50" s="47">
+      <c r="B50" s="1">
         <v>218</v>
       </c>
-      <c r="C50" s="47">
+      <c r="C50" s="1">
         <v>89</v>
       </c>
-      <c r="D50" s="47">
+      <c r="D50" s="1">
         <v>187</v>
       </c>
-      <c r="E50" s="47">
+      <c r="E50" s="1">
         <v>494</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="V15:W15"/>
-    <mergeCell ref="X15:Y15"/>
-    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="B1:AA1"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Z2:AA2"/>
     <mergeCell ref="X3:Y3"/>
     <mergeCell ref="Z3:AA3"/>
     <mergeCell ref="A15:A16"/>
@@ -27277,21 +27284,11 @@
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="B1:AA1"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="T15:U15"/>
+    <mergeCell ref="V15:W15"/>
+    <mergeCell ref="X15:Y15"/>
+    <mergeCell ref="Z15:AA15"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: update NA Bench Forecast — 2026-08-18 13:49
</commit_message>
<xml_diff>
--- a/NA Bench Forecast.xlsx
+++ b/NA Bench Forecast.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbondcrx/Desktop/BOB!/Bench Forecast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6740DF-130B-A347-A39C-345F93944A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C461291-0210-CC42-93EE-44A92F2CA41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="1740" windowWidth="27320" windowHeight="16080" xr2:uid="{25195C4B-21BA-C647-88E3-DB4384B68E18}"/>
+    <workbookView xWindow="30360" yWindow="600" windowWidth="27320" windowHeight="16080" xr2:uid="{25195C4B-21BA-C647-88E3-DB4384B68E18}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench Forecast" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,8 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="528" r:id="rId8"/>
-    <pivotCache cacheId="529" r:id="rId9"/>
+    <pivotCache cacheId="151" r:id="rId8"/>
+    <pivotCache cacheId="155" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="170">
   <si>
     <t>Center</t>
   </si>
@@ -560,6 +560,9 @@
   <si>
     <t>3Q26 WK6</t>
   </si>
+  <si>
+    <t>3Q26 WK7</t>
+  </si>
 </sst>
 </file>
 
@@ -568,7 +571,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -888,7 +891,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1002,9 +1005,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1014,14 +1022,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1029,7 +1036,25 @@
     <cellStyle name="Normal 3" xfId="2" xr:uid="{08B8F7EA-76D3-DF45-B2B8-F681551BBCE4}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -1569,25 +1594,25 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
+                  <c:v>8.4451068057625436E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.2463984103328364E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.8489816194734233E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>6.8554396423248884E-2</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>7.6999503229011432E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>7.7993045206159961E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.9483358171882762E-2</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.9980129160457034E-2</c:v>
+                  <c:v>6.4580228514654739E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.2960755091902635E-2</c:v>
+                  <c:v>7.3025335320417287E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.2960755091902635E-2</c:v>
+                  <c:v>7.6999503229011432E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>8.2960755091902635E-2</c:v>
@@ -2377,9 +2402,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Historic Bench Data'!$Q$24:$Q$107</c:f>
+              <c:f>'Historic Bench Data'!$Q$24:$Q$108</c:f>
               <c:strCache>
-                <c:ptCount val="83"/>
+                <c:ptCount val="84"/>
                 <c:pt idx="0">
                   <c:v>1Q WK 01</c:v>
                 </c:pt>
@@ -2629,15 +2654,18 @@
                 <c:pt idx="82">
                   <c:v>3Q26 WK6</c:v>
                 </c:pt>
+                <c:pt idx="83">
+                  <c:v>3Q26 WK7</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Historic Bench Data'!$R$24:$R$107</c:f>
+              <c:f>'Historic Bench Data'!$R$24:$R$108</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="83"/>
+                <c:ptCount val="84"/>
                 <c:pt idx="0">
                   <c:v>268</c:v>
                 </c:pt>
@@ -2886,6 +2914,9 @@
                 </c:pt>
                 <c:pt idx="82">
                   <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>155</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17770,13 +17801,13 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46241.419074537036" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="83" xr:uid="{C1EC0577-5798-BD42-8B69-BE725BAFED20}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46252.573241550926" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{2AB200AB-C2E2-FD45-A502-66BF023320DC}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="N2:O85" sheet="Historic Bench Data"/>
+    <worksheetSource ref="N2:O86" sheet="Historic Bench Data"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Wk" numFmtId="0">
-      <sharedItems count="101">
+      <sharedItems count="84">
         <s v="1Q WK 01"/>
         <s v="1Q WK 02"/>
         <s v="1Q WK 03"/>
@@ -17860,24 +17891,7 @@
         <s v="3Q26 WK4"/>
         <s v="3Q26 WK5"/>
         <s v="3Q26 WK6"/>
-        <s v="3Q26 WK01" u="1"/>
-        <s v="3Q26 WK02" u="1"/>
-        <s v="3Q26 WK03" u="1"/>
-        <s v="3Q26 WK04" u="1"/>
-        <s v="3Q26 WK05" u="1"/>
-        <s v="3Q26 WK06" u="1"/>
-        <s v="3Q26 WK 01" u="1"/>
-        <s v="3Q26 WK 02" u="1"/>
-        <s v="3Q26 WK 03" u="1"/>
-        <s v="3Q26 WK 04" u="1"/>
-        <s v="3Q26 WK 05" u="1"/>
-        <s v="3Q26 WK 06" u="1"/>
-        <s v="2026 3Q WK 01" u="1"/>
-        <s v="2026 3Q WK 02" u="1"/>
-        <s v="2026 3Q WK 03" u="1"/>
-        <s v="2026 3Q WK 04" u="1"/>
-        <s v="2026 3Q WK 05" u="1"/>
-        <s v="2026 3Q WK 06" u="1"/>
+        <s v="3Q26 WK7"/>
       </sharedItems>
     </cacheField>
     <cacheField name="NA CIC" numFmtId="0">
@@ -17893,7 +17907,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46241.442219097225" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{D3FE744F-E4CE-144D-9062-754059CD7E0E}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46252.573471527779" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{D3FE744F-E4CE-144D-9062-754059CD7E0E}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A30:N33" sheet="Q3 2025"/>
   </cacheSource>
@@ -17906,43 +17920,43 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Wk 01" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="142" maxValue="159"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="159" maxValue="170"/>
     </cacheField>
     <cacheField name="Wk 02" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="148" maxValue="161"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="148" maxValue="166"/>
     </cacheField>
     <cacheField name="Wk 03" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="133" maxValue="161"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="133" maxValue="158"/>
     </cacheField>
     <cacheField name="Wk 04" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="138" maxValue="168"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="138" maxValue="156"/>
     </cacheField>
     <cacheField name="Wk 05" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="121" maxValue="166"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="121" maxValue="152"/>
     </cacheField>
     <cacheField name="Wk 06" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="136" maxValue="180"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="136" maxValue="165"/>
     </cacheField>
     <cacheField name="Wk 07" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="119" maxValue="181"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="119" maxValue="175"/>
     </cacheField>
     <cacheField name="Wk 08" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="114" maxValue="180"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="114" maxValue="176"/>
     </cacheField>
     <cacheField name="Wk 09" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="178"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="172"/>
     </cacheField>
     <cacheField name="Wk 10" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="112" maxValue="212"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="112" maxValue="209"/>
     </cacheField>
     <cacheField name="Wk 11" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="222"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="219"/>
     </cacheField>
     <cacheField name="Wk 12" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="95" maxValue="222"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="95" maxValue="217"/>
     </cacheField>
     <cacheField name="Wk 13" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="218"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="213"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -17954,7 +17968,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="83">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="84">
   <r>
     <x v="0"/>
     <n v="268"/>
@@ -18287,6 +18301,10 @@
     <x v="82"/>
     <n v="144"/>
   </r>
+  <r>
+    <x v="83"/>
+    <n v="155"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
@@ -18294,19 +18312,19 @@
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
   <r>
     <x v="0"/>
-    <n v="142"/>
-    <n v="157"/>
-    <n v="161"/>
-    <n v="168"/>
+    <n v="170"/>
     <n v="166"/>
-    <n v="180"/>
-    <n v="181"/>
-    <n v="180"/>
-    <n v="178"/>
-    <n v="212"/>
-    <n v="222"/>
-    <n v="222"/>
-    <n v="218"/>
+    <n v="158"/>
+    <n v="138"/>
+    <n v="130"/>
+    <n v="147"/>
+    <n v="155"/>
+    <n v="167"/>
+    <n v="172"/>
+    <n v="209"/>
+    <n v="219"/>
+    <n v="217"/>
+    <n v="213"/>
   </r>
   <r>
     <x v="1"/>
@@ -18344,11 +18362,11 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EBC7B274-FD7A-844F-964F-72EF841A0267}" name="PivotTable12" cacheId="528" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
-  <location ref="Q23:R107" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F6FBB504-3C42-4F42-9E28-DCBD3634684A}" name="PivotTable12" cacheId="151" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+  <location ref="Q23:R108" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
-      <items count="102">
+      <items count="85">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -18426,30 +18444,13 @@
         <item x="74"/>
         <item x="75"/>
         <item x="76"/>
-        <item m="1" x="95"/>
-        <item m="1" x="96"/>
-        <item m="1" x="97"/>
-        <item m="1" x="98"/>
-        <item m="1" x="99"/>
-        <item m="1" x="100"/>
-        <item m="1" x="89"/>
-        <item m="1" x="90"/>
-        <item m="1" x="91"/>
-        <item m="1" x="92"/>
-        <item m="1" x="93"/>
-        <item m="1" x="94"/>
-        <item m="1" x="83"/>
-        <item m="1" x="84"/>
-        <item m="1" x="85"/>
-        <item m="1" x="86"/>
-        <item m="1" x="87"/>
-        <item m="1" x="88"/>
         <item x="77"/>
         <item x="78"/>
         <item x="79"/>
         <item x="80"/>
         <item x="81"/>
         <item x="82"/>
+        <item x="83"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -18458,7 +18459,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="84">
+  <rowItems count="85">
     <i>
       <x/>
     </i>
@@ -18691,22 +18692,25 @@
       <x v="76"/>
     </i>
     <i>
-      <x v="95"/>
+      <x v="77"/>
     </i>
     <i>
-      <x v="96"/>
+      <x v="78"/>
     </i>
     <i>
-      <x v="97"/>
+      <x v="79"/>
     </i>
     <i>
-      <x v="98"/>
+      <x v="80"/>
     </i>
     <i>
-      <x v="99"/>
+      <x v="81"/>
     </i>
     <i>
-      <x v="100"/>
+      <x v="82"/>
+    </i>
+    <i>
+      <x v="83"/>
     </i>
     <i t="grand">
       <x/>
@@ -18811,7 +18815,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{04DCFBA1-C6D5-3C43-8822-30BD597F8EAC}" name="PivotTable2" cacheId="529" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="43">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{04DCFBA1-C6D5-3C43-8822-30BD597F8EAC}" name="PivotTable2" cacheId="155" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="43">
   <location ref="A36:E50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisCol" showAll="0">
@@ -18913,7 +18917,7 @@
     <dataField name="  Wk 13" fld="13" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="13">
@@ -18934,23 +18938,23 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="10">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="9">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="8">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -20231,7 +20235,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0E2704-513B-D944-83AA-0507804C032D}">
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1" outlineLevel="1"/>
@@ -20240,7 +20244,7 @@
     <col min="5" max="14" width="10.5" style="1" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -20284,32 +20288,32 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14">
       <c r="A2" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="12">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="C2" s="12">
+        <v>64</v>
+      </c>
+      <c r="D2" s="12">
+        <v>56</v>
+      </c>
+      <c r="E2" s="12">
+        <v>46</v>
+      </c>
+      <c r="F2" s="12">
+        <v>37</v>
+      </c>
+      <c r="G2" s="12">
         <v>44</v>
       </c>
-      <c r="D2" s="12">
-        <v>42</v>
-      </c>
-      <c r="E2" s="12">
-        <v>42</v>
-      </c>
-      <c r="F2" s="12">
-        <v>40</v>
-      </c>
-      <c r="G2" s="12">
-        <v>40</v>
-      </c>
-      <c r="H2" s="8">
-        <v>38</v>
-      </c>
-      <c r="I2" s="8">
+      <c r="H2" s="12">
+        <v>43</v>
+      </c>
+      <c r="I2" s="12">
         <v>38</v>
       </c>
       <c r="J2" s="8">
@@ -20328,32 +20332,32 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14">
       <c r="A3" s="9" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" s="12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" s="12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="12">
         <v>3</v>
       </c>
       <c r="G3" s="12">
-        <v>3</v>
-      </c>
-      <c r="H3" s="11">
-        <v>3</v>
-      </c>
-      <c r="I3" s="11">
+        <v>2</v>
+      </c>
+      <c r="H3" s="12">
+        <v>2</v>
+      </c>
+      <c r="I3" s="12">
         <v>3</v>
       </c>
       <c r="J3" s="11">
@@ -20372,32 +20376,32 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="12">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C4" s="12">
         <v>19</v>
       </c>
       <c r="D4" s="12">
+        <v>19</v>
+      </c>
+      <c r="E4" s="12">
+        <v>18</v>
+      </c>
+      <c r="F4" s="12">
         <v>20</v>
       </c>
-      <c r="E4" s="12">
-        <v>23</v>
-      </c>
-      <c r="F4" s="12">
-        <v>25</v>
-      </c>
       <c r="G4" s="12">
-        <v>25</v>
-      </c>
-      <c r="H4" s="8">
-        <v>27</v>
-      </c>
-      <c r="I4" s="8">
+        <v>26</v>
+      </c>
+      <c r="H4" s="12">
+        <v>41</v>
+      </c>
+      <c r="I4" s="12">
         <v>28</v>
       </c>
       <c r="J4" s="8">
@@ -20416,32 +20420,32 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="12">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C5" s="12">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D5" s="12">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E5" s="12">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="F5" s="12">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G5" s="12">
-        <v>51</v>
-      </c>
-      <c r="H5" s="11">
-        <v>51</v>
-      </c>
-      <c r="I5" s="11">
+        <v>28</v>
+      </c>
+      <c r="H5" s="12">
+        <v>23</v>
+      </c>
+      <c r="I5" s="12">
         <v>49</v>
       </c>
       <c r="J5" s="11">
@@ -20460,32 +20464,32 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6" s="9" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="12">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="12">
+        <v>15</v>
+      </c>
+      <c r="D6" s="12">
+        <v>14</v>
+      </c>
+      <c r="E6" s="12">
+        <v>11</v>
+      </c>
+      <c r="F6" s="12">
+        <v>11</v>
+      </c>
+      <c r="G6" s="12">
         <v>16</v>
       </c>
-      <c r="D6" s="12">
-        <v>16</v>
-      </c>
-      <c r="E6" s="12">
-        <v>17</v>
-      </c>
-      <c r="F6" s="12">
-        <v>17</v>
-      </c>
-      <c r="G6" s="12">
-        <v>18</v>
-      </c>
-      <c r="H6" s="8">
-        <v>17</v>
-      </c>
-      <c r="I6" s="8">
+      <c r="H6" s="12">
+        <v>15</v>
+      </c>
+      <c r="I6" s="12">
         <v>16</v>
       </c>
       <c r="J6" s="8">
@@ -20504,32 +20508,32 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="A7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="12">
+        <v>15</v>
+      </c>
+      <c r="C7" s="12">
         <v>12</v>
       </c>
-      <c r="C7" s="12">
-        <v>14</v>
-      </c>
       <c r="D7" s="12">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E7" s="12">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F7" s="12">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G7" s="12">
-        <v>10</v>
-      </c>
-      <c r="H7" s="11">
+        <v>11</v>
+      </c>
+      <c r="H7" s="12">
         <v>12</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="12">
         <v>13</v>
       </c>
       <c r="J7" s="11">
@@ -20548,7 +20552,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="A8" s="9" t="s">
         <v>20</v>
       </c>
@@ -20570,10 +20574,10 @@
       <c r="G8" s="12">
         <v>20</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="12">
         <v>19</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="12">
         <v>20</v>
       </c>
       <c r="J8" s="8">
@@ -20592,37 +20596,37 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="6">
         <f>SUM(B2:B8)</f>
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C9" s="6">
         <f t="shared" ref="C9:N9" si="0">SUM(C2:C8)</f>
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D9" s="6">
         <f t="shared" si="0"/>
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E9" s="6">
         <f t="shared" si="0"/>
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="F9" s="6">
         <f t="shared" si="0"/>
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="G9" s="6">
         <f t="shared" si="0"/>
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="H9" s="6">
         <f t="shared" si="0"/>
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
@@ -20649,37 +20653,37 @@
         <v>213</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="7">
         <f>+B9/$B$11</f>
-        <v>6.8554396423248884E-2</v>
+        <v>8.4451068057625436E-2</v>
       </c>
       <c r="C10" s="7">
         <f t="shared" ref="C10:N10" si="1">+C9/$B$11</f>
-        <v>7.6999503229011432E-2</v>
+        <v>8.2463984103328364E-2</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
-        <v>7.7993045206159961E-2</v>
+        <v>7.8489816194734233E-2</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9483358171882762E-2</v>
+        <v>6.8554396423248884E-2</v>
       </c>
       <c r="F10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9980129160457034E-2</v>
+        <v>6.4580228514654739E-2</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" si="1"/>
-        <v>8.2960755091902635E-2</v>
+        <v>7.3025335320417287E-2</v>
       </c>
       <c r="H10" s="7">
         <f t="shared" si="1"/>
-        <v>8.2960755091902635E-2</v>
+        <v>7.6999503229011432E-2</v>
       </c>
       <c r="I10" s="7">
         <f t="shared" si="1"/>
@@ -20706,7 +20710,7 @@
         <v>0.10581222056631892</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -20715,47 +20719,47 @@
       </c>
       <c r="C11" s="10"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="N14"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="N15"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="N16">
         <v>136</v>
       </c>
     </row>
-    <row r="17" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="14:14">
       <c r="N17">
         <v>180</v>
       </c>
     </row>
-    <row r="18" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="14:14">
       <c r="N18">
         <f>+N17-N16</f>
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="14:14">
       <c r="N19"/>
     </row>
-    <row r="20" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="14:14">
       <c r="N20"/>
     </row>
-    <row r="21" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="14:14">
       <c r="N21"/>
     </row>
-    <row r="22" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="14:14">
       <c r="N22"/>
     </row>
-    <row r="23" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="14:14">
       <c r="N23"/>
     </row>
-    <row r="24" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="14:14">
       <c r="N24"/>
     </row>
-    <row r="25" spans="14:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="14:14">
       <c r="N25"/>
     </row>
   </sheetData>
@@ -20767,8 +20771,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE199676-AB11-A54D-A3E4-E1A2A649D0A0}">
-  <dimension ref="A1:R107"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:R108"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -20781,10 +20785,10 @@
     <col min="10" max="10" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="32">
       <c r="A1" s="13" t="s">
         <v>24</v>
       </c>
@@ -20822,7 +20826,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15">
       <c r="A2" s="14">
         <v>2025</v>
       </c>
@@ -20868,7 +20872,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15">
       <c r="A3" s="14">
         <v>2025</v>
       </c>
@@ -20914,7 +20918,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15">
       <c r="A4" s="14">
         <v>2025</v>
       </c>
@@ -20960,7 +20964,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15">
       <c r="A5" s="14">
         <v>2025</v>
       </c>
@@ -21006,7 +21010,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15">
       <c r="A6" s="14">
         <v>2025</v>
       </c>
@@ -21052,7 +21056,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="A7" s="14">
         <v>2025</v>
       </c>
@@ -21098,7 +21102,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15">
       <c r="A8" s="14">
         <v>2025</v>
       </c>
@@ -21144,7 +21148,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15">
       <c r="A9" s="14">
         <v>2025</v>
       </c>
@@ -21190,7 +21194,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15">
       <c r="A10" s="14">
         <v>2025</v>
       </c>
@@ -21236,7 +21240,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15">
       <c r="A11" s="14">
         <v>2025</v>
       </c>
@@ -21282,7 +21286,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15">
       <c r="A12" s="14">
         <v>2025</v>
       </c>
@@ -21328,7 +21332,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15">
       <c r="A13" s="14">
         <v>2025</v>
       </c>
@@ -21374,7 +21378,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15">
       <c r="A14" s="14">
         <v>2025</v>
       </c>
@@ -21420,7 +21424,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15">
       <c r="A15" s="14">
         <v>2025</v>
       </c>
@@ -21466,7 +21470,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15">
       <c r="A16" s="14">
         <v>2025</v>
       </c>
@@ -21512,7 +21516,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18">
       <c r="A17" s="14">
         <v>2025</v>
       </c>
@@ -21558,7 +21562,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18">
       <c r="A18" s="14">
         <v>2025</v>
       </c>
@@ -21604,7 +21608,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18">
       <c r="A19" s="14">
         <v>2025</v>
       </c>
@@ -21650,7 +21654,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18">
       <c r="A20" s="14">
         <v>2025</v>
       </c>
@@ -21696,7 +21700,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18">
       <c r="A21" s="14">
         <v>2025</v>
       </c>
@@ -21742,7 +21746,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18">
       <c r="A22" s="14">
         <v>2025</v>
       </c>
@@ -21788,7 +21792,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18">
       <c r="A23" s="14">
         <v>2025</v>
       </c>
@@ -21840,7 +21844,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18">
       <c r="A24" s="14">
         <v>2025</v>
       </c>
@@ -21888,11 +21892,11 @@
       <c r="Q24" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="R24">
+      <c r="R24" s="47">
         <v>268</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18">
       <c r="A25" s="14">
         <v>2025</v>
       </c>
@@ -21940,11 +21944,11 @@
       <c r="Q25" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="R25">
+      <c r="R25" s="47">
         <v>290</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18">
       <c r="A26" s="14">
         <v>2025</v>
       </c>
@@ -21992,11 +21996,11 @@
       <c r="Q26" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="R26">
+      <c r="R26" s="47">
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18">
       <c r="A27" s="14">
         <v>2025</v>
       </c>
@@ -22044,11 +22048,11 @@
       <c r="Q27" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="R27">
+      <c r="R27" s="47">
         <v>228</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18">
       <c r="A28" s="14">
         <v>2025</v>
       </c>
@@ -22096,11 +22100,11 @@
       <c r="Q28" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="R28">
+      <c r="R28" s="47">
         <v>214</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18">
       <c r="A29" s="14">
         <v>2025</v>
       </c>
@@ -22148,11 +22152,11 @@
       <c r="Q29" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="R29">
+      <c r="R29" s="47">
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18">
       <c r="A30" s="14">
         <v>2025</v>
       </c>
@@ -22200,11 +22204,11 @@
       <c r="Q30" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="R30">
+      <c r="R30" s="47">
         <v>207</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18">
       <c r="A31" s="14">
         <v>2025</v>
       </c>
@@ -22252,11 +22256,11 @@
       <c r="Q31" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="R31">
+      <c r="R31" s="47">
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18">
       <c r="A32" s="14">
         <v>2025</v>
       </c>
@@ -22304,11 +22308,11 @@
       <c r="Q32" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="R32">
+      <c r="R32" s="47">
         <v>189</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18">
       <c r="A33" s="14">
         <v>2025</v>
       </c>
@@ -22355,11 +22359,11 @@
       <c r="Q33" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="R33">
+      <c r="R33" s="47">
         <v>180</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18">
       <c r="A34" s="14">
         <v>2025</v>
       </c>
@@ -22406,11 +22410,11 @@
       <c r="Q34" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="R34">
+      <c r="R34" s="47">
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18">
       <c r="A35" s="14">
         <v>2025</v>
       </c>
@@ -22458,11 +22462,11 @@
       <c r="Q35" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="R35">
+      <c r="R35" s="47">
         <v>154</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18">
       <c r="A36" s="14">
         <v>2025</v>
       </c>
@@ -22509,11 +22513,11 @@
       <c r="Q36" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="R36">
+      <c r="R36" s="47">
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18">
       <c r="A37" s="14">
         <v>2025</v>
       </c>
@@ -22560,11 +22564,11 @@
       <c r="Q37" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="R37">
+      <c r="R37" s="47">
         <v>169</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18">
       <c r="A38" s="14">
         <v>2025</v>
       </c>
@@ -22611,11 +22615,11 @@
       <c r="Q38" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="R38">
+      <c r="R38" s="47">
         <v>142</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18">
       <c r="A39" s="14">
         <v>2025</v>
       </c>
@@ -22662,11 +22666,11 @@
       <c r="Q39" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="R39">
+      <c r="R39" s="47">
         <v>169</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18">
       <c r="A40" s="14">
         <v>2025</v>
       </c>
@@ -22713,11 +22717,11 @@
       <c r="Q40" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="R40">
+      <c r="R40" s="47">
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18">
       <c r="A41" s="14">
         <v>2025</v>
       </c>
@@ -22765,11 +22769,11 @@
       <c r="Q41" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R41">
+      <c r="R41" s="47">
         <v>164</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18">
       <c r="A42" s="14">
         <v>2025</v>
       </c>
@@ -22817,11 +22821,11 @@
       <c r="Q42" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="R42">
+      <c r="R42" s="47">
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18">
       <c r="A43" s="14">
         <v>2025</v>
       </c>
@@ -22869,11 +22873,11 @@
       <c r="Q43" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="R43">
+      <c r="R43" s="47">
         <v>147</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18">
       <c r="A44" s="14">
         <v>2025</v>
       </c>
@@ -22921,11 +22925,11 @@
       <c r="Q44" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="R44">
+      <c r="R44" s="47">
         <v>146</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18">
       <c r="A45" s="14">
         <v>2025</v>
       </c>
@@ -22973,11 +22977,11 @@
       <c r="Q45" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="R45">
+      <c r="R45" s="47">
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18">
       <c r="A46" s="14">
         <v>2025</v>
       </c>
@@ -23025,11 +23029,11 @@
       <c r="Q46" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="R46">
+      <c r="R46" s="47">
         <v>161</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18">
       <c r="A47" s="14">
         <v>2025</v>
       </c>
@@ -23077,11 +23081,11 @@
       <c r="Q47" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="R47">
+      <c r="R47" s="47">
         <v>159</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18">
       <c r="A48" s="14">
         <v>2025</v>
       </c>
@@ -23129,11 +23133,11 @@
       <c r="Q48" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="R48">
+      <c r="R48" s="47">
         <v>133</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18">
       <c r="A49" s="14">
         <v>2025</v>
       </c>
@@ -23181,11 +23185,11 @@
       <c r="Q49" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="R49">
+      <c r="R49" s="47">
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18">
       <c r="A50" s="14">
         <v>2025</v>
       </c>
@@ -23233,11 +23237,11 @@
       <c r="Q50" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="R50">
+      <c r="R50" s="47">
         <v>181</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18">
       <c r="A51" s="14">
         <v>2025</v>
       </c>
@@ -23285,11 +23289,11 @@
       <c r="Q51" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="R51">
+      <c r="R51" s="47">
         <v>177</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18">
       <c r="A52" s="14">
         <v>2025</v>
       </c>
@@ -23337,11 +23341,11 @@
       <c r="Q52" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="R52">
+      <c r="R52" s="47">
         <v>165</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18">
       <c r="A53" s="14">
         <v>2025</v>
       </c>
@@ -23389,11 +23393,11 @@
       <c r="Q53" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="R53">
+      <c r="R53" s="47">
         <v>168</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18">
       <c r="A54" s="14">
         <v>2026</v>
       </c>
@@ -23441,11 +23445,11 @@
       <c r="Q54" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="R54">
+      <c r="R54" s="47">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18">
       <c r="A55" s="14">
         <v>2026</v>
       </c>
@@ -23493,11 +23497,11 @@
       <c r="Q55" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="R55">
+      <c r="R55" s="47">
         <v>156</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18">
       <c r="A56" s="14">
         <v>2026</v>
       </c>
@@ -23545,11 +23549,11 @@
       <c r="Q56" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="R56">
+      <c r="R56" s="47">
         <v>158</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:18">
       <c r="A57" s="14">
         <v>2026</v>
       </c>
@@ -23597,11 +23601,11 @@
       <c r="Q57" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="R57">
+      <c r="R57" s="47">
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:18">
       <c r="A58" s="14">
         <v>2026</v>
       </c>
@@ -23649,11 +23653,11 @@
       <c r="Q58" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="R58">
+      <c r="R58" s="47">
         <v>128</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:18">
       <c r="A59" s="14">
         <v>2026</v>
       </c>
@@ -23701,11 +23705,11 @@
       <c r="Q59" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="R59">
+      <c r="R59" s="47">
         <v>134</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:18">
       <c r="A60" s="14">
         <v>2026</v>
       </c>
@@ -23753,11 +23757,11 @@
       <c r="Q60" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="R60">
+      <c r="R60" s="47">
         <v>123</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:18">
       <c r="A61" s="14">
         <v>2026</v>
       </c>
@@ -23805,11 +23809,11 @@
       <c r="Q61" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="R61">
+      <c r="R61" s="47">
         <v>123</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:18">
       <c r="A62" s="14">
         <v>2026</v>
       </c>
@@ -23857,11 +23861,11 @@
       <c r="Q62" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="R62">
+      <c r="R62" s="47">
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:18">
       <c r="A63" s="14">
         <v>2026</v>
       </c>
@@ -23909,11 +23913,11 @@
       <c r="Q63" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="R63">
+      <c r="R63" s="47">
         <v>119</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:18">
       <c r="A64" s="14">
         <v>2026</v>
       </c>
@@ -23961,11 +23965,11 @@
       <c r="Q64" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="R64">
+      <c r="R64" s="47">
         <v>107</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:18">
       <c r="A65" s="14">
         <v>2026</v>
       </c>
@@ -24013,11 +24017,11 @@
       <c r="Q65" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="R65">
+      <c r="R65" s="47">
         <v>110</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:18">
       <c r="A66" s="14">
         <v>2026</v>
       </c>
@@ -24064,11 +24068,11 @@
       <c r="Q66" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="R66">
+      <c r="R66" s="47">
         <v>137</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:18">
       <c r="A67" s="14">
         <v>2026</v>
       </c>
@@ -24115,11 +24119,11 @@
       <c r="Q67" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="R67">
+      <c r="R67" s="47">
         <v>124</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:18">
       <c r="A68" s="14">
         <v>2026</v>
       </c>
@@ -24166,11 +24170,11 @@
       <c r="Q68" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="R68">
+      <c r="R68" s="47">
         <v>127</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:18">
       <c r="A69" s="14">
         <v>2026</v>
       </c>
@@ -24217,11 +24221,11 @@
       <c r="Q69" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="R69">
+      <c r="R69" s="47">
         <v>101</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:18">
       <c r="A70" s="14">
         <v>2026</v>
       </c>
@@ -24269,11 +24273,11 @@
       <c r="Q70" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="R70">
+      <c r="R70" s="47">
         <v>116</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:18">
       <c r="A71" s="14">
         <v>2026</v>
       </c>
@@ -24328,11 +24332,11 @@
       <c r="Q71" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="R71">
+      <c r="R71" s="47">
         <v>124</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:18">
       <c r="A72" s="14">
         <v>2026</v>
       </c>
@@ -24380,11 +24384,11 @@
       <c r="Q72" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="R72">
+      <c r="R72" s="47">
         <v>134</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="17" thickBot="1">
       <c r="A73" s="14">
         <v>2026</v>
       </c>
@@ -24439,11 +24443,11 @@
       <c r="Q73" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="R73">
+      <c r="R73" s="47">
         <v>113</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="18" thickTop="1" thickBot="1">
       <c r="A74" s="14">
         <v>2026</v>
       </c>
@@ -24491,11 +24495,11 @@
       <c r="Q74" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="R74">
+      <c r="R74" s="47">
         <v>118</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="18" thickTop="1" thickBot="1">
       <c r="A75" s="14">
         <v>2026</v>
       </c>
@@ -24550,11 +24554,11 @@
       <c r="Q75" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="R75">
+      <c r="R75" s="47">
         <v>127</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:18">
       <c r="A76" s="14">
         <v>2026</v>
       </c>
@@ -24602,11 +24606,11 @@
       <c r="Q76" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="R76">
+      <c r="R76" s="47">
         <v>231</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:18">
       <c r="A77" s="14">
         <v>2026</v>
       </c>
@@ -24661,11 +24665,11 @@
       <c r="Q77" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="R77">
+      <c r="R77" s="47">
         <v>201</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:18">
       <c r="A78" s="14">
         <v>2026</v>
       </c>
@@ -24712,11 +24716,11 @@
       <c r="Q78" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="R78">
+      <c r="R78" s="47">
         <v>180</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:18">
       <c r="A79" s="14">
         <v>2026</v>
       </c>
@@ -24752,7 +24756,7 @@
         <v>176</v>
       </c>
       <c r="L79" t="str">
-        <f t="shared" ref="L79:L84" si="9">+B79&amp;" "&amp;C79</f>
+        <f t="shared" ref="L79:L85" si="9">+B79&amp;" "&amp;C79</f>
         <v>3Q WK 01</v>
       </c>
       <c r="N79" t="s">
@@ -24764,11 +24768,11 @@
       <c r="Q79" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="R79">
+      <c r="R79" s="47">
         <v>171</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:18">
       <c r="A80" s="14">
         <v>2026</v>
       </c>
@@ -24800,7 +24804,7 @@
         <v>19</v>
       </c>
       <c r="K80" s="15">
-        <f t="shared" ref="K80:K84" si="10">SUM(D80:J80)</f>
+        <f t="shared" ref="K80:K85" si="10">SUM(D80:J80)</f>
         <v>165</v>
       </c>
       <c r="L80" t="str">
@@ -24816,11 +24820,11 @@
       <c r="Q80" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="R80">
+      <c r="R80" s="47">
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:18">
       <c r="A81" s="14">
         <v>2026</v>
       </c>
@@ -24868,11 +24872,11 @@
       <c r="Q81" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="R81">
+      <c r="R81" s="47">
         <v>143</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:18">
       <c r="A82" s="14">
         <v>2026</v>
       </c>
@@ -24920,11 +24924,11 @@
       <c r="Q82" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="R82">
+      <c r="R82" s="47">
         <v>114</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:18">
       <c r="A83" s="14">
         <v>2026</v>
       </c>
@@ -24972,11 +24976,11 @@
       <c r="Q83" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="R83">
+      <c r="R83" s="47">
         <v>110</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:18">
       <c r="A84" s="14">
         <v>2026</v>
       </c>
@@ -25024,11 +25028,49 @@
       <c r="Q84" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="R84">
+      <c r="R84" s="47">
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:18">
+      <c r="A85" s="14">
+        <v>2026</v>
+      </c>
+      <c r="B85" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C85" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D85" s="16">
+        <v>43</v>
+      </c>
+      <c r="E85" s="16">
+        <v>15</v>
+      </c>
+      <c r="F85" s="16">
+        <v>12</v>
+      </c>
+      <c r="G85" s="16">
+        <v>2</v>
+      </c>
+      <c r="H85" s="16">
+        <v>23</v>
+      </c>
+      <c r="I85" s="16">
+        <v>19</v>
+      </c>
+      <c r="J85" s="16">
+        <v>41</v>
+      </c>
+      <c r="K85" s="15">
+        <f t="shared" si="10"/>
+        <v>155</v>
+      </c>
+      <c r="L85" t="str">
+        <f t="shared" si="9"/>
+        <v>3Q WK 07</v>
+      </c>
       <c r="N85" t="s">
         <v>168</v>
       </c>
@@ -25038,184 +25080,198 @@
       <c r="Q85" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="R85">
+      <c r="R85" s="47">
         <v>101</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:18">
+      <c r="N86" t="s">
+        <v>169</v>
+      </c>
+      <c r="O86">
+        <v>155</v>
+      </c>
       <c r="Q86" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="R86">
+      <c r="R86" s="47">
         <v>78</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:18">
       <c r="Q87" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="R87">
+      <c r="R87" s="47">
         <v>73</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:18">
       <c r="Q88" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="R88">
+      <c r="R88" s="47">
         <v>121</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:18">
       <c r="Q89" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="R89">
+      <c r="R89" s="47">
         <v>117</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:18">
       <c r="Q90" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="R90">
+      <c r="R90" s="47">
         <v>114</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:18">
       <c r="Q91" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="R91">
+      <c r="R91" s="47">
         <v>114</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:18">
       <c r="Q92" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="R92">
+      <c r="R92" s="47">
         <v>114</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:18">
       <c r="Q93" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="R93">
+      <c r="R93" s="47">
         <v>137</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:18">
       <c r="Q94" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="R94">
+      <c r="R94" s="47">
         <v>126</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:18">
       <c r="Q95" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="R95">
+      <c r="R95" s="47">
         <v>151</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:18">
       <c r="Q96" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="R96">
+      <c r="R96" s="47">
         <v>125</v>
       </c>
     </row>
-    <row r="97" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="97" spans="17:18">
       <c r="Q97" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="R97">
+      <c r="R97" s="47">
         <v>116</v>
       </c>
     </row>
-    <row r="98" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="98" spans="17:18">
       <c r="Q98" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="R98">
+      <c r="R98" s="47">
         <v>145</v>
       </c>
     </row>
-    <row r="99" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="99" spans="17:18">
       <c r="Q99" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="R99">
+      <c r="R99" s="47">
         <v>148</v>
       </c>
     </row>
-    <row r="100" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="100" spans="17:18">
       <c r="Q100" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="R100">
+      <c r="R100" s="47">
         <v>152</v>
       </c>
     </row>
-    <row r="101" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="101" spans="17:18">
       <c r="Q101" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="R101">
+      <c r="R101" s="47">
         <v>176</v>
       </c>
     </row>
-    <row r="102" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="102" spans="17:18">
       <c r="Q102" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="R102">
+      <c r="R102" s="47">
         <v>165</v>
       </c>
     </row>
-    <row r="103" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="103" spans="17:18">
       <c r="Q103" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="R103">
+      <c r="R103" s="47">
         <v>160</v>
       </c>
     </row>
-    <row r="104" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="104" spans="17:18">
       <c r="Q104" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="R104">
+      <c r="R104" s="47">
         <v>138</v>
       </c>
     </row>
-    <row r="105" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="105" spans="17:18">
       <c r="Q105" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="R105">
+      <c r="R105" s="47">
         <v>132</v>
       </c>
     </row>
-    <row r="106" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="106" spans="17:18">
       <c r="Q106" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="R106">
+      <c r="R106" s="47">
         <v>144</v>
       </c>
     </row>
-    <row r="107" spans="17:18" x14ac:dyDescent="0.2">
+    <row r="107" spans="17:18">
       <c r="Q107" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="R107" s="47">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="108" spans="17:18">
+      <c r="Q108" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="R107">
-        <v>12387</v>
+      <c r="R108" s="47">
+        <v>12542</v>
       </c>
     </row>
   </sheetData>
@@ -25228,7 +25284,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56B9C08D-E3AB-A84E-BFC7-CB4DF670EA2E}">
   <dimension ref="A1:AA50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
@@ -25237,151 +25293,151 @@
     <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27">
       <c r="A1" s="21"/>
-      <c r="B1" s="45" t="s">
+      <c r="B1" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="46"/>
-      <c r="AA1" s="46"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
+      <c r="AA1" s="42"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A2" s="44" t="s">
+    <row r="2" spans="1:27">
+      <c r="A2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="42" t="s">
+      <c r="C2" s="45"/>
+      <c r="D2" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="43"/>
-      <c r="F2" s="42" t="s">
+      <c r="E2" s="45"/>
+      <c r="F2" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="43"/>
-      <c r="H2" s="42" t="s">
+      <c r="G2" s="45"/>
+      <c r="H2" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="I2" s="43"/>
-      <c r="J2" s="42" t="s">
+      <c r="I2" s="45"/>
+      <c r="J2" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="K2" s="43"/>
-      <c r="L2" s="42" t="s">
+      <c r="K2" s="45"/>
+      <c r="L2" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="M2" s="43"/>
-      <c r="N2" s="42" t="s">
+      <c r="M2" s="45"/>
+      <c r="N2" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="O2" s="43"/>
-      <c r="P2" s="42" t="s">
+      <c r="O2" s="45"/>
+      <c r="P2" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="Q2" s="43"/>
-      <c r="R2" s="42" t="s">
+      <c r="Q2" s="45"/>
+      <c r="R2" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="S2" s="43"/>
-      <c r="T2" s="42" t="s">
+      <c r="S2" s="45"/>
+      <c r="T2" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="U2" s="43"/>
-      <c r="V2" s="42" t="s">
+      <c r="U2" s="45"/>
+      <c r="V2" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="W2" s="43"/>
-      <c r="X2" s="42" t="s">
+      <c r="W2" s="45"/>
+      <c r="X2" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="Y2" s="43"/>
-      <c r="Z2" s="42" t="s">
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="AA2" s="43"/>
+      <c r="AA2" s="45"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="44"/>
-      <c r="B3" s="42" t="s">
+    <row r="3" spans="1:27">
+      <c r="A3" s="43"/>
+      <c r="B3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="42" t="s">
+      <c r="C3" s="45"/>
+      <c r="D3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="42" t="s">
+      <c r="E3" s="45"/>
+      <c r="F3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="42" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="I3" s="43"/>
-      <c r="J3" s="42" t="s">
+      <c r="I3" s="45"/>
+      <c r="J3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="K3" s="43"/>
-      <c r="L3" s="42" t="s">
+      <c r="K3" s="45"/>
+      <c r="L3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="M3" s="43"/>
-      <c r="N3" s="42" t="s">
+      <c r="M3" s="45"/>
+      <c r="N3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="O3" s="43"/>
-      <c r="P3" s="42" t="s">
+      <c r="O3" s="45"/>
+      <c r="P3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="42" t="s">
+      <c r="Q3" s="45"/>
+      <c r="R3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="S3" s="43"/>
-      <c r="T3" s="42" t="s">
+      <c r="S3" s="45"/>
+      <c r="T3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="U3" s="43"/>
-      <c r="V3" s="42" t="s">
+      <c r="U3" s="45"/>
+      <c r="V3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="W3" s="43"/>
-      <c r="X3" s="42" t="s">
+      <c r="W3" s="45"/>
+      <c r="X3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="42" t="s">
+      <c r="Y3" s="45"/>
+      <c r="Z3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="AA3" s="43"/>
+      <c r="AA3" s="45"/>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="44"/>
+    <row r="4" spans="1:27">
+      <c r="A4" s="43"/>
       <c r="B4" s="23" t="s">
         <v>142</v>
       </c>
@@ -25461,7 +25517,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27">
       <c r="A5" s="21" t="s">
         <v>14</v>
       </c>
@@ -25544,7 +25600,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27">
       <c r="A6" s="21" t="s">
         <v>18</v>
       </c>
@@ -25627,7 +25683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27">
       <c r="A7" s="21" t="s">
         <v>19</v>
       </c>
@@ -25710,7 +25766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27">
       <c r="A8" s="21" t="s">
         <v>15</v>
       </c>
@@ -25793,7 +25849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
@@ -25876,7 +25932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27">
       <c r="A10" s="21" t="s">
         <v>20</v>
       </c>
@@ -25959,7 +26015,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27">
       <c r="A11" s="21" t="s">
         <v>16</v>
       </c>
@@ -26042,7 +26098,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27">
       <c r="A13" s="25" t="s">
         <v>144</v>
       </c>
@@ -26125,8 +26181,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A15" s="44" t="s">
+    <row r="15" spans="1:27">
+      <c r="A15" s="43" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="22" t="s">
@@ -26169,21 +26225,21 @@
         <v>140</v>
       </c>
       <c r="O15" s="36"/>
-      <c r="P15" s="41"/>
-      <c r="Q15" s="41"/>
-      <c r="R15" s="41"/>
-      <c r="S15" s="41"/>
-      <c r="T15" s="41"/>
-      <c r="U15" s="41"/>
-      <c r="V15" s="41"/>
-      <c r="W15" s="41"/>
-      <c r="X15" s="41"/>
-      <c r="Y15" s="41"/>
-      <c r="Z15" s="41"/>
-      <c r="AA15" s="41"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="46"/>
+      <c r="Y15" s="46"/>
+      <c r="Z15" s="46"/>
+      <c r="AA15" s="46"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A16" s="44"/>
+    <row r="16" spans="1:27">
+      <c r="A16" s="43"/>
       <c r="B16" s="23" t="s">
         <v>143</v>
       </c>
@@ -26236,7 +26292,7 @@
       <c r="Z16" s="31"/>
       <c r="AA16" s="32"/>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:27">
       <c r="A17" s="21" t="s">
         <v>14</v>
       </c>
@@ -26305,7 +26361,7 @@
       <c r="Z17" s="33"/>
       <c r="AA17" s="32"/>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:27">
       <c r="A18" s="21" t="s">
         <v>18</v>
       </c>
@@ -26374,7 +26430,7 @@
       <c r="Z18" s="33"/>
       <c r="AA18" s="32"/>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:27">
       <c r="A19" s="21" t="s">
         <v>19</v>
       </c>
@@ -26443,7 +26499,7 @@
       <c r="Z19" s="33"/>
       <c r="AA19" s="32"/>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:27">
       <c r="A20" s="21" t="s">
         <v>15</v>
       </c>
@@ -26512,7 +26568,7 @@
       <c r="Z20" s="33"/>
       <c r="AA20" s="32"/>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:27">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
@@ -26581,7 +26637,7 @@
       <c r="Z21" s="33"/>
       <c r="AA21" s="32"/>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:27">
       <c r="A22" s="21" t="s">
         <v>20</v>
       </c>
@@ -26650,7 +26706,7 @@
       <c r="Z22" s="33"/>
       <c r="AA22" s="32"/>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:27">
       <c r="A23" s="21" t="s">
         <v>16</v>
       </c>
@@ -26719,7 +26775,7 @@
       <c r="Z23" s="33"/>
       <c r="AA23" s="32"/>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:27">
       <c r="A24" s="35"/>
       <c r="N24" s="37"/>
       <c r="P24" s="32"/>
@@ -26735,7 +26791,7 @@
       <c r="Z24" s="32"/>
       <c r="AA24" s="32"/>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:27">
       <c r="A25" s="25" t="s">
         <v>144</v>
       </c>
@@ -26804,7 +26860,7 @@
       <c r="Z25" s="34"/>
       <c r="AA25" s="32"/>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:27">
       <c r="A30" s="27" t="s">
         <v>145</v>
       </c>
@@ -26848,37 +26904,37 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:27">
       <c r="A31" s="2" t="s">
         <v>146</v>
       </c>
       <c r="B31" s="1">
         <f>+'Bench Forecast'!B9</f>
-        <v>138</v>
+        <v>170</v>
       </c>
       <c r="C31" s="1">
         <f>+'Bench Forecast'!C9</f>
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="D31" s="1">
         <f>+'Bench Forecast'!D9</f>
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E31" s="1">
         <f>+'Bench Forecast'!E9</f>
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="F31" s="1">
         <f>+'Bench Forecast'!F9</f>
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="G31" s="1">
         <f>+'Bench Forecast'!G9</f>
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="H31" s="1">
         <f>+'Bench Forecast'!H9</f>
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="I31" s="1">
         <f>+'Bench Forecast'!I9</f>
@@ -26905,7 +26961,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:27">
       <c r="A32" s="2" t="s">
         <v>147</v>
       </c>
@@ -26962,7 +27018,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14">
       <c r="A33" s="2" t="s">
         <v>148</v>
       </c>
@@ -27006,7 +27062,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14">
       <c r="B36" s="39" t="s">
         <v>149</v>
       </c>
@@ -27014,7 +27070,7 @@
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14">
       <c r="A37" s="38" t="s">
         <v>150</v>
       </c>
@@ -27031,229 +27087,248 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14">
       <c r="A38" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B38" s="1">
-        <v>142</v>
-      </c>
-      <c r="C38" s="1">
+      <c r="B38" s="48">
+        <v>170</v>
+      </c>
+      <c r="C38" s="48">
         <v>159</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="48">
         <v>159</v>
       </c>
-      <c r="E38" s="1">
-        <v>460</v>
+      <c r="E38" s="48">
+        <v>488</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14">
       <c r="A39" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B39" s="1">
-        <v>157</v>
-      </c>
-      <c r="C39" s="1">
+      <c r="B39" s="48">
+        <v>166</v>
+      </c>
+      <c r="C39" s="48">
         <v>148</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="48">
         <v>161</v>
       </c>
-      <c r="E39" s="1">
-        <v>466</v>
+      <c r="E39" s="48">
+        <v>475</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14">
       <c r="A40" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B40" s="1">
-        <v>161</v>
-      </c>
-      <c r="C40" s="1">
+      <c r="B40" s="48">
+        <v>158</v>
+      </c>
+      <c r="C40" s="48">
         <v>133</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="48">
         <v>154</v>
       </c>
-      <c r="E40" s="1">
-        <v>448</v>
+      <c r="E40" s="48">
+        <v>445</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14">
       <c r="A41" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B41" s="1">
-        <v>168</v>
-      </c>
-      <c r="C41" s="1">
+      <c r="B41" s="48">
         <v>138</v>
       </c>
-      <c r="D41" s="1">
+      <c r="C41" s="48">
+        <v>138</v>
+      </c>
+      <c r="D41" s="48">
         <v>156</v>
       </c>
-      <c r="E41" s="1">
-        <v>462</v>
+      <c r="E41" s="48">
+        <v>432</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14">
       <c r="A42" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B42" s="1">
-        <v>166</v>
-      </c>
-      <c r="C42" s="1">
+      <c r="B42" s="48">
+        <v>130</v>
+      </c>
+      <c r="C42" s="48">
         <v>121</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="48">
         <v>152</v>
       </c>
-      <c r="E42" s="1">
-        <v>439</v>
+      <c r="E42" s="48">
+        <v>403</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14">
       <c r="A43" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B43" s="1">
-        <v>180</v>
-      </c>
-      <c r="C43" s="1">
+      <c r="B43" s="48">
+        <v>147</v>
+      </c>
+      <c r="C43" s="48">
         <v>136</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="48">
         <v>165</v>
       </c>
-      <c r="E43" s="1">
-        <v>481</v>
+      <c r="E43" s="48">
+        <v>448</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14">
       <c r="A44" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B44" s="1">
-        <v>181</v>
-      </c>
-      <c r="C44" s="1">
+      <c r="B44" s="48">
+        <v>155</v>
+      </c>
+      <c r="C44" s="48">
         <v>119</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="48">
         <v>175</v>
       </c>
-      <c r="E44" s="1">
-        <v>475</v>
+      <c r="E44" s="48">
+        <v>449</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14">
       <c r="A45" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B45" s="1">
-        <v>180</v>
-      </c>
-      <c r="C45" s="1">
+      <c r="B45" s="48">
+        <v>167</v>
+      </c>
+      <c r="C45" s="48">
         <v>114</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="48">
         <v>176</v>
       </c>
-      <c r="E45" s="1">
-        <v>470</v>
+      <c r="E45" s="48">
+        <v>457</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14">
       <c r="A46" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B46" s="1">
-        <v>178</v>
-      </c>
-      <c r="C46" s="1">
+      <c r="B46" s="48">
+        <v>172</v>
+      </c>
+      <c r="C46" s="48">
         <v>104</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="48">
         <v>171</v>
       </c>
-      <c r="E46" s="1">
-        <v>453</v>
+      <c r="E46" s="48">
+        <v>447</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14">
       <c r="A47" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B47" s="1">
-        <v>212</v>
-      </c>
-      <c r="C47" s="1">
+      <c r="B47" s="48">
+        <v>209</v>
+      </c>
+      <c r="C47" s="48">
         <v>112</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="48">
         <v>196</v>
       </c>
-      <c r="E47" s="1">
-        <v>520</v>
+      <c r="E47" s="48">
+        <v>517</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14">
       <c r="A48" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B48" s="1">
-        <v>222</v>
-      </c>
-      <c r="C48" s="1">
+      <c r="B48" s="48">
+        <v>219</v>
+      </c>
+      <c r="C48" s="48">
         <v>98</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="48">
         <v>192</v>
       </c>
-      <c r="E48" s="1">
-        <v>512</v>
+      <c r="E48" s="48">
+        <v>509</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5">
       <c r="A49" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B49" s="1">
-        <v>222</v>
-      </c>
-      <c r="C49" s="1">
+      <c r="B49" s="48">
+        <v>217</v>
+      </c>
+      <c r="C49" s="48">
         <v>95</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="48">
         <v>191</v>
       </c>
-      <c r="E49" s="1">
-        <v>508</v>
+      <c r="E49" s="48">
+        <v>503</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5">
       <c r="A50" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B50" s="1">
-        <v>218</v>
-      </c>
-      <c r="C50" s="1">
+      <c r="B50" s="48">
+        <v>213</v>
+      </c>
+      <c r="C50" s="48">
         <v>89</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="48">
         <v>187</v>
       </c>
-      <c r="E50" s="1">
-        <v>494</v>
+      <c r="E50" s="48">
+        <v>489</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="V15:W15"/>
+    <mergeCell ref="X15:Y15"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="T15:U15"/>
     <mergeCell ref="B1:AA1"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:C2"/>
@@ -27270,25 +27345,6 @@
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="Z2:AA2"/>
     <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="T3:U3"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="V15:W15"/>
-    <mergeCell ref="X15:Y15"/>
-    <mergeCell ref="Z15:AA15"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>